<commit_message>
@basit-eSpark R1 DNP kr dia ha BOM me.
</commit_message>
<xml_diff>
--- a/Design Files/Design-v2.1.1/PowerBackup-v2.1.1/BOM/Client_BOM.xlsx
+++ b/Design Files/Design-v2.1.1/PowerBackup-v2.1.1/BOM/Client_BOM.xlsx
@@ -1,15 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\issamsmaali-powerbackupcircuit\Design Files\Design-v2.1.1\PowerBackup-v2.1.1\BOM\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="19635" windowHeight="7620"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19635" windowHeight="7620"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -27,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="327">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="327">
   <si>
     <t>#</t>
   </si>
@@ -1013,14 +1018,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="26">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1032,14 +1031,14 @@
       <sz val="10"/>
       <color indexed="13"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1047,175 +1046,41 @@
       <sz val="10"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <strike/>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="18"/>
-      <color theme="3"/>
+      <strike/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1234,194 +1099,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="16">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -1512,253 +1191,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1795,11 +1232,11 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1807,68 +1244,36 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="0003A4CB"/>
-      <color rgb="002CD0B2"/>
+      <color rgb="FF03A4CB"/>
+      <color rgb="FF2CD0B2"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -2126,28 +1531,29 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K72"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="3.14285714285714" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.7142857142857" style="1" customWidth="1"/>
+    <col min="2" max="2" width="3.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="1" customWidth="1"/>
     <col min="4" max="4" width="36" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="26.5714285714286" customWidth="1"/>
-    <col min="7" max="7" width="33.4285714285714" customWidth="1"/>
-    <col min="8" max="8" width="21.4285714285714" customWidth="1"/>
-    <col min="9" max="9" width="17.8571428571429" customWidth="1"/>
-    <col min="10" max="10" width="16.7142857142857" customWidth="1"/>
-    <col min="11" max="11" width="29.4285714285714" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" customWidth="1"/>
+    <col min="9" max="9" width="17.85546875" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" customWidth="1"/>
+    <col min="11" max="11" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" spans="1:11">
+    <row r="1" spans="1:11">
       <c r="A1" s="2"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2156,11 +1562,11 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-    </row>
-    <row r="2" ht="15.75" spans="1:11">
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+    </row>
+    <row r="2" spans="1:11">
       <c r="A2" s="2"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -2196,7 +1602,7 @@
     <row r="3" spans="1:11">
       <c r="A3" s="2"/>
       <c r="B3" s="7">
-        <f>ROW(B3)-ROW($B$2)</f>
+        <f t="shared" ref="B3:B34" si="0">ROW(B3)-ROW($B$2)</f>
         <v>1</v>
       </c>
       <c r="C3" s="8" t="s">
@@ -2225,10 +1631,10 @@
       </c>
       <c r="K3" s="9"/>
     </row>
-    <row r="4" ht="24.75" spans="1:11">
+    <row r="4" spans="1:11" ht="24">
       <c r="A4" s="2"/>
       <c r="B4" s="7">
-        <f>ROW(B4)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="C4" s="8" t="s">
@@ -2260,7 +1666,7 @@
     <row r="5" spans="1:11">
       <c r="A5" s="2"/>
       <c r="B5" s="7">
-        <f>ROW(B5)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="C5" s="8" t="s">
@@ -2289,10 +1695,10 @@
       </c>
       <c r="K5" s="9"/>
     </row>
-    <row r="6" ht="24.75" spans="1:11">
+    <row r="6" spans="1:11" ht="24">
       <c r="A6" s="2"/>
       <c r="B6" s="7">
-        <f>ROW(B6)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C6" s="8" t="s">
@@ -2324,7 +1730,7 @@
     <row r="7" spans="1:11">
       <c r="A7" s="2"/>
       <c r="B7" s="7">
-        <f>ROW(B7)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C7" s="8" t="s">
@@ -2353,10 +1759,10 @@
       </c>
       <c r="K7" s="9"/>
     </row>
-    <row r="8" ht="24.75" spans="1:11">
+    <row r="8" spans="1:11" ht="24">
       <c r="A8" s="2"/>
       <c r="B8" s="7">
-        <f>ROW(B8)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C8" s="8" t="s">
@@ -2385,10 +1791,10 @@
       </c>
       <c r="K8" s="11"/>
     </row>
-    <row r="9" ht="24.75" spans="1:11">
+    <row r="9" spans="1:11" ht="36">
       <c r="A9" s="2"/>
       <c r="B9" s="7">
-        <f>ROW(B9)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C9" s="8" t="s">
@@ -2420,7 +1826,7 @@
     <row r="10" spans="1:11">
       <c r="A10" s="2"/>
       <c r="B10" s="7">
-        <f>ROW(B10)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C10" s="8" t="s">
@@ -2452,7 +1858,7 @@
     <row r="11" spans="1:11">
       <c r="A11" s="2"/>
       <c r="B11" s="7">
-        <f>ROW(B11)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C11" s="8" t="s">
@@ -2481,10 +1887,10 @@
       </c>
       <c r="K11" s="9"/>
     </row>
-    <row r="12" ht="24.75" spans="1:11">
+    <row r="12" spans="1:11" ht="24">
       <c r="A12" s="2"/>
       <c r="B12" s="7">
-        <f>ROW(B12)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C12" s="8" t="s">
@@ -2513,10 +1919,10 @@
       </c>
       <c r="K12" s="11"/>
     </row>
-    <row r="13" ht="24.75" spans="1:11">
+    <row r="13" spans="1:11" ht="24">
       <c r="A13" s="2"/>
       <c r="B13" s="7">
-        <f>ROW(B13)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C13" s="8" t="s">
@@ -2545,10 +1951,10 @@
       </c>
       <c r="K13" s="9"/>
     </row>
-    <row r="14" ht="24.75" spans="1:11">
+    <row r="14" spans="1:11" ht="24">
       <c r="A14" s="2"/>
       <c r="B14" s="7">
-        <f>ROW(B14)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C14" s="8" t="s">
@@ -2577,10 +1983,10 @@
       </c>
       <c r="K14" s="11"/>
     </row>
-    <row r="15" ht="24.75" spans="1:11">
+    <row r="15" spans="1:11" ht="24">
       <c r="A15" s="2"/>
       <c r="B15" s="7">
-        <f>ROW(B15)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C15" s="8" t="s">
@@ -2612,7 +2018,7 @@
     <row r="16" spans="1:11">
       <c r="A16" s="2"/>
       <c r="B16" s="7">
-        <f>ROW(B16)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C16" s="8" t="s">
@@ -2640,7 +2046,7 @@
     <row r="17" spans="1:11">
       <c r="A17" s="2"/>
       <c r="B17" s="7">
-        <f>ROW(B17)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="C17" s="8" t="s">
@@ -2672,7 +2078,7 @@
     <row r="18" spans="1:11">
       <c r="A18" s="2"/>
       <c r="B18" s="7">
-        <f>ROW(B18)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="C18" s="8" t="s">
@@ -2704,7 +2110,7 @@
     <row r="19" spans="1:11">
       <c r="A19" s="2"/>
       <c r="B19" s="7">
-        <f>ROW(B19)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="C19" s="8" t="s">
@@ -2736,7 +2142,7 @@
     <row r="20" spans="1:11">
       <c r="A20" s="2"/>
       <c r="B20" s="7">
-        <f>ROW(B20)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C20" s="8" t="s">
@@ -2768,7 +2174,7 @@
     <row r="21" spans="1:11">
       <c r="A21" s="2"/>
       <c r="B21" s="7">
-        <f>ROW(B21)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="C21" s="8" t="s">
@@ -2797,10 +2203,10 @@
       </c>
       <c r="K21" s="9"/>
     </row>
-    <row r="22" ht="15.75" spans="1:11">
+    <row r="22" spans="1:11">
       <c r="A22" s="2"/>
       <c r="B22" s="7">
-        <f>ROW(B22)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="C22" s="8" t="s">
@@ -2829,10 +2235,10 @@
       </c>
       <c r="K22" s="11"/>
     </row>
-    <row r="23" ht="24.75" spans="1:11">
+    <row r="23" spans="1:11" ht="24">
       <c r="A23" s="2"/>
       <c r="B23" s="7">
-        <f>ROW(B23)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="C23" s="8" t="s">
@@ -2861,10 +2267,10 @@
       </c>
       <c r="K23" s="9"/>
     </row>
-    <row r="24" ht="24.75" spans="1:11">
+    <row r="24" spans="1:11" ht="24">
       <c r="A24" s="2"/>
       <c r="B24" s="7">
-        <f>ROW(B24)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="C24" s="8" t="s">
@@ -2893,10 +2299,10 @@
       </c>
       <c r="K24" s="11"/>
     </row>
-    <row r="25" ht="15.75" spans="1:11">
+    <row r="25" spans="1:11">
       <c r="A25" s="2"/>
       <c r="B25" s="7">
-        <f>ROW(B25)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="C25" s="8" t="s">
@@ -2928,7 +2334,7 @@
     <row r="26" spans="1:11">
       <c r="A26" s="2"/>
       <c r="B26" s="7">
-        <f>ROW(B26)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="C26" s="8" t="s">
@@ -2957,10 +2363,10 @@
       </c>
       <c r="K26" s="11"/>
     </row>
-    <row r="27" ht="36.75" spans="1:11">
+    <row r="27" spans="1:11" ht="36">
       <c r="A27" s="2"/>
       <c r="B27" s="7">
-        <f>ROW(B27)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="C27" s="8" t="s">
@@ -2992,7 +2398,7 @@
     <row r="28" spans="1:11">
       <c r="A28" s="2"/>
       <c r="B28" s="7">
-        <f>ROW(B28)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="C28" s="8" t="s">
@@ -3021,10 +2427,10 @@
       </c>
       <c r="K28" s="11"/>
     </row>
-    <row r="29" ht="24.75" spans="1:11">
+    <row r="29" spans="1:11" ht="24">
       <c r="A29" s="2"/>
       <c r="B29" s="7">
-        <f>ROW(B29)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="C29" s="8" t="s">
@@ -3053,10 +2459,10 @@
       </c>
       <c r="K29" s="9"/>
     </row>
-    <row r="30" ht="24.75" spans="1:11">
+    <row r="30" spans="1:11" ht="24">
       <c r="A30" s="2"/>
       <c r="B30" s="7">
-        <f>ROW(B30)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="C30" s="13" t="s">
@@ -3085,10 +2491,10 @@
       </c>
       <c r="K30" s="11"/>
     </row>
-    <row r="31" ht="24.75" spans="1:11">
+    <row r="31" spans="1:11" ht="24">
       <c r="A31" s="2"/>
       <c r="B31" s="7">
-        <f>ROW(B31)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>29</v>
       </c>
       <c r="C31" s="8" t="s">
@@ -3109,7 +2515,7 @@
       <c r="H31" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="I31" s="15" t="s">
+      <c r="I31" s="14" t="s">
         <v>109</v>
       </c>
       <c r="J31" s="9">
@@ -3117,10 +2523,10 @@
       </c>
       <c r="K31" s="9"/>
     </row>
-    <row r="32" ht="24.75" spans="1:11">
+    <row r="32" spans="1:11" ht="24">
       <c r="A32" s="2"/>
       <c r="B32" s="7">
-        <f>ROW(B32)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C32" s="8" t="s">
@@ -3141,7 +2547,7 @@
       <c r="H32" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="I32" s="15" t="s">
+      <c r="I32" s="14" t="s">
         <v>109</v>
       </c>
       <c r="J32" s="11">
@@ -3152,7 +2558,7 @@
     <row r="33" spans="1:11">
       <c r="A33" s="2"/>
       <c r="B33" s="7">
-        <f>ROW(B33)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>31</v>
       </c>
       <c r="C33" s="8" t="s">
@@ -3173,7 +2579,7 @@
       <c r="H33" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="I33" s="15" t="s">
+      <c r="I33" s="14" t="s">
         <v>109</v>
       </c>
       <c r="J33" s="9">
@@ -3181,10 +2587,10 @@
       </c>
       <c r="K33" s="9"/>
     </row>
-    <row r="34" ht="24.75" spans="1:11">
+    <row r="34" spans="1:11" ht="24">
       <c r="A34" s="2"/>
       <c r="B34" s="7">
-        <f>ROW(B34)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C34" s="8" t="s">
@@ -3205,7 +2611,7 @@
       <c r="H34" s="11" t="s">
         <v>161</v>
       </c>
-      <c r="I34" s="15" t="s">
+      <c r="I34" s="14" t="s">
         <v>109</v>
       </c>
       <c r="J34" s="11">
@@ -3213,10 +2619,10 @@
       </c>
       <c r="K34" s="11"/>
     </row>
-    <row r="35" ht="15.75" spans="1:11">
+    <row r="35" spans="1:11">
       <c r="A35" s="2"/>
       <c r="B35" s="7">
-        <f>ROW(B35)-ROW($B$2)</f>
+        <f t="shared" ref="B35:B66" si="1">ROW(B35)-ROW($B$2)</f>
         <v>33</v>
       </c>
       <c r="C35" s="13" t="s">
@@ -3233,7 +2639,7 @@
       </c>
       <c r="G35" s="10"/>
       <c r="H35" s="9"/>
-      <c r="I35" s="15" t="s">
+      <c r="I35" s="14" t="s">
         <v>109</v>
       </c>
       <c r="J35" s="9">
@@ -3241,10 +2647,10 @@
       </c>
       <c r="K35" s="9"/>
     </row>
-    <row r="36" ht="15.75" spans="1:11">
+    <row r="36" spans="1:11">
       <c r="A36" s="2"/>
       <c r="B36" s="7">
-        <f>ROW(B36)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>34</v>
       </c>
       <c r="C36" s="13" t="s">
@@ -3265,7 +2671,7 @@
       <c r="H36" s="11" t="s">
         <v>170</v>
       </c>
-      <c r="I36" s="15" t="s">
+      <c r="I36" s="14" t="s">
         <v>109</v>
       </c>
       <c r="J36" s="11">
@@ -3273,42 +2679,44 @@
       </c>
       <c r="K36" s="11"/>
     </row>
-    <row r="37" ht="36.75" spans="1:11">
+    <row r="37" spans="1:11" ht="36">
       <c r="A37" s="2"/>
       <c r="B37" s="7">
-        <f>ROW(B37)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>35</v>
       </c>
       <c r="C37" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="D37" s="9" t="s">
+      <c r="D37" s="19" t="s">
         <v>172</v>
       </c>
-      <c r="E37" s="10" t="s">
+      <c r="E37" s="20" t="s">
         <v>173</v>
       </c>
-      <c r="F37" s="9" t="s">
+      <c r="F37" s="19" t="s">
         <v>174</v>
       </c>
-      <c r="G37" s="10" t="s">
+      <c r="G37" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="H37" s="9" t="s">
+      <c r="H37" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="I37" s="10" t="s">
+      <c r="I37" s="20" t="s">
         <v>176</v>
       </c>
-      <c r="J37" s="9">
-        <v>1</v>
-      </c>
-      <c r="K37" s="9"/>
+      <c r="J37" s="19">
+        <v>1</v>
+      </c>
+      <c r="K37" s="21" t="s">
+        <v>277</v>
+      </c>
     </row>
     <row r="38" spans="1:11">
       <c r="A38" s="2"/>
       <c r="B38" s="7">
-        <f>ROW(B38)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>36</v>
       </c>
       <c r="C38" s="8" t="s">
@@ -3340,7 +2748,7 @@
     <row r="39" spans="1:11">
       <c r="A39" s="2"/>
       <c r="B39" s="7">
-        <f>ROW(B39)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>37</v>
       </c>
       <c r="C39" s="8" t="s">
@@ -3372,7 +2780,7 @@
     <row r="40" spans="1:11">
       <c r="A40" s="2"/>
       <c r="B40" s="7">
-        <f>ROW(B40)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>38</v>
       </c>
       <c r="C40" s="8" t="s">
@@ -3404,7 +2812,7 @@
     <row r="41" spans="1:11">
       <c r="A41" s="2"/>
       <c r="B41" s="7">
-        <f>ROW(B41)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>39</v>
       </c>
       <c r="C41" s="8" t="s">
@@ -3433,10 +2841,10 @@
       </c>
       <c r="K41" s="9"/>
     </row>
-    <row r="42" ht="24.75" spans="1:11">
+    <row r="42" spans="1:11" ht="24">
       <c r="A42" s="2"/>
       <c r="B42" s="7">
-        <f>ROW(B42)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>40</v>
       </c>
       <c r="C42" s="8" t="s">
@@ -3468,7 +2876,7 @@
     <row r="43" spans="1:11">
       <c r="A43" s="2"/>
       <c r="B43" s="7">
-        <f>ROW(B43)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>41</v>
       </c>
       <c r="C43" s="8" t="s">
@@ -3500,7 +2908,7 @@
     <row r="44" spans="1:11">
       <c r="A44" s="2"/>
       <c r="B44" s="7">
-        <f>ROW(B44)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>42</v>
       </c>
       <c r="C44" s="8" t="s">
@@ -3532,7 +2940,7 @@
     <row r="45" spans="1:11">
       <c r="A45" s="2"/>
       <c r="B45" s="7">
-        <f>ROW(B45)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>43</v>
       </c>
       <c r="C45" s="8" t="s">
@@ -3564,7 +2972,7 @@
     <row r="46" spans="1:11">
       <c r="A46" s="2"/>
       <c r="B46" s="7">
-        <f>ROW(B46)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>44</v>
       </c>
       <c r="C46" s="8" t="s">
@@ -3589,10 +2997,10 @@
       </c>
       <c r="K46" s="11"/>
     </row>
-    <row r="47" ht="24.75" spans="1:11">
+    <row r="47" spans="1:11" ht="24">
       <c r="A47" s="2"/>
       <c r="B47" s="7">
-        <f>ROW(B47)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>45</v>
       </c>
       <c r="C47" s="8" t="s">
@@ -3621,10 +3029,10 @@
       </c>
       <c r="K47" s="9"/>
     </row>
-    <row r="48" ht="36.75" spans="1:11">
+    <row r="48" spans="1:11" ht="36">
       <c r="A48" s="2"/>
       <c r="B48" s="7">
-        <f>ROW(B48)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>46</v>
       </c>
       <c r="C48" s="8" t="s">
@@ -3653,10 +3061,10 @@
       </c>
       <c r="K48" s="11"/>
     </row>
-    <row r="49" ht="24.75" spans="1:11">
+    <row r="49" spans="1:11" ht="24">
       <c r="A49" s="2"/>
       <c r="B49" s="7">
-        <f>ROW(B49)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>47</v>
       </c>
       <c r="C49" s="8" t="s">
@@ -3688,7 +3096,7 @@
     <row r="50" spans="1:11">
       <c r="A50" s="2"/>
       <c r="B50" s="7">
-        <f>ROW(B50)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>48</v>
       </c>
       <c r="C50" s="8" t="s">
@@ -3720,7 +3128,7 @@
     <row r="51" spans="1:11">
       <c r="A51" s="2"/>
       <c r="B51" s="7">
-        <f>ROW(B51)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>49</v>
       </c>
       <c r="C51" s="8" t="s">
@@ -3752,7 +3160,7 @@
     <row r="52" spans="1:11">
       <c r="A52" s="2"/>
       <c r="B52" s="7">
-        <f>ROW(B52)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>50</v>
       </c>
       <c r="C52" s="8" t="s">
@@ -3784,7 +3192,7 @@
     <row r="53" spans="1:11">
       <c r="A53" s="2"/>
       <c r="B53" s="7">
-        <f>ROW(B53)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>51</v>
       </c>
       <c r="C53" s="8" t="s">
@@ -3816,7 +3224,7 @@
     <row r="54" spans="1:11">
       <c r="A54" s="2"/>
       <c r="B54" s="7">
-        <f>ROW(B54)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>52</v>
       </c>
       <c r="C54" s="8" t="s">
@@ -3848,7 +3256,7 @@
     <row r="55" spans="1:11">
       <c r="A55" s="2"/>
       <c r="B55" s="7">
-        <f>ROW(B55)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>53</v>
       </c>
       <c r="C55" s="8" t="s">
@@ -3880,7 +3288,7 @@
     <row r="56" spans="1:11">
       <c r="A56" s="2"/>
       <c r="B56" s="7">
-        <f>ROW(B56)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>54</v>
       </c>
       <c r="C56" s="8" t="s">
@@ -3912,7 +3320,7 @@
     <row r="57" spans="1:11">
       <c r="A57" s="2"/>
       <c r="B57" s="7">
-        <f>ROW(B57)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>55</v>
       </c>
       <c r="C57" s="8" t="s">
@@ -3944,7 +3352,7 @@
     <row r="58" spans="1:11">
       <c r="A58" s="2"/>
       <c r="B58" s="7">
-        <f>ROW(B58)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>56</v>
       </c>
       <c r="C58" s="8" t="s">
@@ -3973,10 +3381,10 @@
       </c>
       <c r="K58" s="11"/>
     </row>
-    <row r="59" ht="24.75" spans="1:11">
+    <row r="59" spans="1:11" ht="24">
       <c r="A59" s="2"/>
       <c r="B59" s="7">
-        <f>ROW(B59)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>57</v>
       </c>
       <c r="C59" s="8" t="s">
@@ -4008,7 +3416,7 @@
     <row r="60" spans="1:11">
       <c r="A60" s="2"/>
       <c r="B60" s="7">
-        <f>ROW(B60)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>58</v>
       </c>
       <c r="C60" s="8" t="s">
@@ -4040,7 +3448,7 @@
     <row r="61" spans="1:11">
       <c r="A61" s="2"/>
       <c r="B61" s="7">
-        <f>ROW(B61)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>59</v>
       </c>
       <c r="C61" s="8" t="s">
@@ -4072,41 +3480,41 @@
     <row r="62" spans="1:11">
       <c r="A62" s="2"/>
       <c r="B62" s="7">
-        <f>ROW(B62)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>60</v>
       </c>
       <c r="C62" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="D62" s="11" t="s">
+      <c r="D62" s="17" t="s">
         <v>276</v>
       </c>
-      <c r="E62" s="12" t="s">
+      <c r="E62" s="16" t="s">
         <v>254</v>
       </c>
-      <c r="F62" s="11" t="s">
+      <c r="F62" s="17" t="s">
         <v>241</v>
       </c>
-      <c r="G62" s="12" t="s">
+      <c r="G62" s="16" t="s">
         <v>255</v>
       </c>
-      <c r="H62" s="11" t="s">
+      <c r="H62" s="17" t="s">
         <v>102</v>
       </c>
       <c r="I62" s="16" t="s">
         <v>277</v>
       </c>
-      <c r="J62" s="11">
-        <v>1</v>
-      </c>
-      <c r="K62" s="17" t="s">
+      <c r="J62" s="17">
+        <v>1</v>
+      </c>
+      <c r="K62" s="18" t="s">
         <v>277</v>
       </c>
     </row>
     <row r="63" spans="1:11">
       <c r="A63" s="2"/>
       <c r="B63" s="7">
-        <f>ROW(B63)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>61</v>
       </c>
       <c r="C63" s="8" t="s">
@@ -4135,10 +3543,10 @@
       </c>
       <c r="K63" s="9"/>
     </row>
-    <row r="64" ht="24.75" spans="1:11">
+    <row r="64" spans="1:11" ht="36">
       <c r="A64" s="2"/>
       <c r="B64" s="7">
-        <f>ROW(B64)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>62</v>
       </c>
       <c r="C64" s="13" t="s">
@@ -4167,10 +3575,10 @@
       </c>
       <c r="K64" s="11"/>
     </row>
-    <row r="65" ht="24.75" spans="1:11">
+    <row r="65" spans="1:11" ht="24">
       <c r="A65" s="2"/>
       <c r="B65" s="7">
-        <f>ROW(B65)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>63</v>
       </c>
       <c r="C65" s="13" t="s">
@@ -4199,10 +3607,10 @@
       </c>
       <c r="K65" s="9"/>
     </row>
-    <row r="66" ht="24.75" spans="1:11">
+    <row r="66" spans="1:11" ht="24">
       <c r="A66" s="2"/>
       <c r="B66" s="7">
-        <f>ROW(B66)-ROW($B$2)</f>
+        <f t="shared" si="1"/>
         <v>64</v>
       </c>
       <c r="C66" s="13" t="s">
@@ -4234,7 +3642,7 @@
     <row r="67" spans="1:11">
       <c r="A67" s="2"/>
       <c r="B67" s="7">
-        <f>ROW(B67)-ROW($B$2)</f>
+        <f t="shared" ref="B67:B72" si="2">ROW(B67)-ROW($B$2)</f>
         <v>65</v>
       </c>
       <c r="C67" s="13" t="s">
@@ -4263,10 +3671,10 @@
       </c>
       <c r="K67" s="9"/>
     </row>
-    <row r="68" ht="24.75" spans="1:11">
+    <row r="68" spans="1:11" ht="24">
       <c r="A68" s="2"/>
       <c r="B68" s="7">
-        <f>ROW(B68)-ROW($B$2)</f>
+        <f t="shared" si="2"/>
         <v>66</v>
       </c>
       <c r="C68" s="13" t="s">
@@ -4295,10 +3703,10 @@
       </c>
       <c r="K68" s="11"/>
     </row>
-    <row r="69" ht="24.75" spans="1:11">
+    <row r="69" spans="1:11" ht="24">
       <c r="A69" s="2"/>
       <c r="B69" s="7">
-        <f>ROW(B69)-ROW($B$2)</f>
+        <f t="shared" si="2"/>
         <v>67</v>
       </c>
       <c r="C69" s="13" t="s">
@@ -4327,10 +3735,10 @@
       </c>
       <c r="K69" s="9"/>
     </row>
-    <row r="70" ht="24.75" spans="1:11">
+    <row r="70" spans="1:11" ht="24">
       <c r="A70" s="2"/>
       <c r="B70" s="7">
-        <f>ROW(B70)-ROW($B$2)</f>
+        <f t="shared" si="2"/>
         <v>68</v>
       </c>
       <c r="C70" s="13" t="s">
@@ -4362,7 +3770,7 @@
     <row r="71" spans="1:11">
       <c r="A71" s="2"/>
       <c r="B71" s="7">
-        <f>ROW(B71)-ROW($B$2)</f>
+        <f t="shared" si="2"/>
         <v>69</v>
       </c>
       <c r="C71" s="13" t="s">
@@ -4391,10 +3799,10 @@
       </c>
       <c r="K71" s="9"/>
     </row>
-    <row r="72" ht="36.75" spans="1:11">
+    <row r="72" spans="1:11" ht="36">
       <c r="A72" s="2"/>
       <c r="B72" s="7">
-        <f>ROW(B72)-ROW($B$2)</f>
+        <f t="shared" si="2"/>
         <v>70</v>
       </c>
       <c r="C72" s="13" t="s">
@@ -4429,6 +3837,5 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>